<commit_message>
feat: dịch quest + story_dialogue phong cách tự nhiên (bình thường)
- Dịch lại 17,463 dòng quest với phong cách tiếng Việt tự nhiên
- Dịch 119,492 dòng story_dialogue (hội thoại, cốt truyện, phụ đề)
- Cập nhật prompts: lore, quest, story_dialogue (bỏ văn phong Hán-Việt)
- Thêm domain story_dialogue vào translate_gemini_gemma_parallel.py
- Sync toàn bộ bản dịch vào SQLite DBs
- Patch TiengViet_99_P_direct_patch.pak (35 segments)
</commit_message>
<xml_diff>
--- a/mistral_translate_work/split_by_prompt/excel/name_title/lang_bag/lang_bag__name_title__part_0001.xlsx
+++ b/mistral_translate_work/split_by_prompt/excel/name_title/lang_bag/lang_bag__name_title__part_0001.xlsx
@@ -2,13 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="translation" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'translation'!$A$1:$N$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -25,23 +28,23 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,33 +52,21 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -440,6 +431,22 @@
   </sheetPr>
   <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="80" customWidth="1" min="12" max="12"/>
+    <col width="80" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -514,216 +521,217 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>NAME_TITLE_0000068</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>name_title</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>name_title_prompt.md</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>lang_bag.json</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>lang_bag.db</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>ItemMainType</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Id</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>ui</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Weapon</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Vũ khí</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>keep_proper_name</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>NAME_TITLE_0000069</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>name_title</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>name_title_prompt.md</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>lang_bag.json</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>lang_bag.db</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>ItemMainType</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Id</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>ui</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Echo</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Echo</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>keep_glossary_term</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>NAME_TITLE_0000070</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>name_title</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>name_title_prompt.md</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>lang_bag.json</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>lang_bag.db</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>ItemMainType</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Id</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>ui</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Missions</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Nhiệm vụ</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Missions</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>keep_proper_name</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A1:N4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>